<commit_message>
Update REITs map for 2026-10-23 list and confirmed listings
</commit_message>
<xml_diff>
--- a/REITs_location_updating.xlsx
+++ b/REITs_location_updating.xlsx
@@ -2662,7 +2662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -6902,6 +6902,147 @@
         </is>
       </c>
     </row>
+    <row r="91" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">180505.SZ</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中金杭州安居宁巢</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">杭州市城市建设投资集团有限公司</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">杭州市明石公寓项目</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">基础设施REITs</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">保障性租赁住房</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">杭州市</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">浙江省</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{杭州市明石公寓项目}</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">180702.SZ</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">银华粤海水务水利</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">广东粤海控股集团有限公司</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">飞来峡项目，潮州项目</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">基础设施REITs</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水利基础设施</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">清远市，潮州市</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">广东省，广东省</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{飞来峡项目}|{潮州项目}</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">508095.SH</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国泰海通中建租赁住房</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中国建筑集团有限公司</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中建·幸孚+公寓（上海松江店）</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">基础设施REITs</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">保障性租赁住房</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上海市</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上海市</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{中建·幸孚+公寓（上海松江店）}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6910,7 +7051,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -7792,17 +7933,17 @@
       <c r="A21"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">国泰海通中国建筑租赁住房</t>
+          <t xml:space="preserve">中金菜鸟仓储物流</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">中国建筑集团有限公司</t>
+          <t xml:space="preserve">阿里巴巴集团</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">中建·幸孚+公寓（上海松江店）</t>
+          <t xml:space="preserve">嘉兴传云项目，嘉兴传祥项目</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -7812,22 +7953,22 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">保障性租赁住房</t>
+          <t xml:space="preserve">仓储物流基础设施</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">上海市</t>
+          <t xml:space="preserve">嘉兴市</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">上海市</t>
+          <t xml:space="preserve">浙江省</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t xml:space="preserve">{中建·幸孚+公寓（上海松江店）}</t>
+          <t xml:space="preserve">{嘉兴传云项目，嘉兴传祥项目}</t>
         </is>
       </c>
     </row>
@@ -7835,42 +7976,42 @@
       <c r="A22"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">银华粤海水务水利</t>
+          <t xml:space="preserve">中金开元旅业</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">广东粤海控股集团有限公司</t>
+          <t xml:space="preserve">Taeway Real Estate Limited（香港）</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">飞来峡项目，潮州项目</t>
+          <t xml:space="preserve">杭州开元名都项目、温州开元名都项目、嵊州开元名都项目</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">基础设施REITs</t>
+          <t xml:space="preserve">商业不动产REITs</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">水利基础设施</t>
+          <t xml:space="preserve">酒店</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">清远市，潮州市</t>
+          <t xml:space="preserve">杭州市，温州市，绍兴市</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve">广东省，广东省</t>
+          <t xml:space="preserve">浙江省，浙江省，浙江省</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t xml:space="preserve">{飞来峡项目}|{潮州项目}</t>
+          <t xml:space="preserve">{杭州开元名都项目}|{温州开元名都项目}|{嵊州开元名都项目}</t>
         </is>
       </c>
     </row>
@@ -7878,42 +8019,42 @@
       <c r="A23"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">中金菜鸟仓储物流</t>
+          <t xml:space="preserve">华夏华润置地</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">阿里巴巴集团</t>
+          <t xml:space="preserve">华润（集团）有限公司</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">嘉兴传云项目，嘉兴传祥项目</t>
+          <t xml:space="preserve">南通万象城、临沂万象汇</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">基础设施REITs</t>
+          <t xml:space="preserve">商业不动产REITs</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">仓储物流基础设施</t>
+          <t xml:space="preserve">商业零售</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">嘉兴市</t>
+          <t xml:space="preserve">南通市，临沂市</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">浙江省</t>
+          <t xml:space="preserve">江苏省，山东省</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t xml:space="preserve">{嘉兴传云项目，嘉兴传祥项目}</t>
+          <t xml:space="preserve">{南通万象城}|{临沂万象汇}</t>
         </is>
       </c>
     </row>
@@ -7921,17 +8062,17 @@
       <c r="A24"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">中金开元旅业</t>
+          <t xml:space="preserve">红土创新茂业</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Taeway Real Estate Limited（香港）</t>
+          <t xml:space="preserve">深圳茂业（集团）股份有限公司</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭州开元名都项目、温州开元名都项目、嵊州开元名都项目</t>
+          <t xml:space="preserve">成都市茂业中心C塔项目</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -7941,22 +8082,22 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">酒店</t>
+          <t xml:space="preserve">办公</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭州市，温州市，绍兴市</t>
+          <t xml:space="preserve">成都市</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">浙江省，浙江省，浙江省</t>
+          <t xml:space="preserve">四川省</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t xml:space="preserve">{杭州开元名都项目}|{温州开元名都项目}|{嵊州开元名都项目}</t>
+          <t xml:space="preserve">{成都市茂业中心C塔项目}</t>
         </is>
       </c>
     </row>
@@ -7964,42 +8105,42 @@
       <c r="A25"/>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">华夏华润置地</t>
+          <t xml:space="preserve">长城华能燃煤发电</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">华润（集团）有限公司</t>
+          <t xml:space="preserve">华能国际电力股份有限公司</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">南通万象城、临沂万象汇</t>
+          <t xml:space="preserve">华能青岛项目</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业不动产REITs</t>
+          <t xml:space="preserve">基础设施REITs</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业零售</t>
+          <t xml:space="preserve">能源基础设施</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">南通市，临沂市</t>
+          <t xml:space="preserve">青岛市</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">江苏省，山东省</t>
+          <t xml:space="preserve">山东省</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t xml:space="preserve">{南通万象城}|{临沂万象汇}</t>
+          <t xml:space="preserve">{华能青岛项目}</t>
         </is>
       </c>
     </row>
@@ -8007,42 +8148,42 @@
       <c r="A26"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">红土创新茂业</t>
+          <t xml:space="preserve">华夏华润电力燃煤发电</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">深圳茂业（集团）股份有限公司</t>
+          <t xml:space="preserve">华润电力控股有限公司</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">成都市茂业中心C塔项目</t>
+          <t xml:space="preserve">华润焦作电厂项目</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业不动产REITs</t>
+          <t xml:space="preserve">基础设施REITs</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">办公</t>
+          <t xml:space="preserve">能源基础设施</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">成都市</t>
+          <t xml:space="preserve">焦作市</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">四川省</t>
+          <t xml:space="preserve">河南省</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t xml:space="preserve">{成都市茂业中心C塔项目}</t>
+          <t xml:space="preserve">{华润焦作电厂项目}</t>
         </is>
       </c>
     </row>
@@ -8050,17 +8191,17 @@
       <c r="A27"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">中金杭州安居保障性租赁住房</t>
+          <t xml:space="preserve">华夏蜀道集团高速公路</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭州市城市建设投资集团有限公司</t>
+          <t xml:space="preserve">蜀道投资集团有限责任公司</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭州市明石公寓项目</t>
+          <t xml:space="preserve">雅泸高速公路项目</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -8070,22 +8211,22 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">保障性租赁住房</t>
+          <t xml:space="preserve">交通基础设施</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭州市</t>
+          <t xml:space="preserve">雅安市，凉山彝族自治州</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">浙江省</t>
+          <t xml:space="preserve">四川省，四川省</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t xml:space="preserve">{杭州市明石公寓项目}</t>
+          <t xml:space="preserve">{雅泸高速公路项目}|{雅泸高速公路项目}</t>
         </is>
       </c>
     </row>
@@ -8093,17 +8234,17 @@
       <c r="A28"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">长城华能燃煤发电</t>
+          <t xml:space="preserve">华夏龙岗城投产业园</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">华能国际电力股份有限公司</t>
+          <t xml:space="preserve">深圳市龙岗区城市建设投资集团有限公司</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">华能青岛项目</t>
+          <t xml:space="preserve">智慧家园项目</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -8113,22 +8254,22 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">能源基础设施</t>
+          <t xml:space="preserve">园区基础设施</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">青岛市</t>
+          <t xml:space="preserve">深圳市</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">山东省</t>
+          <t xml:space="preserve">广东省</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t xml:space="preserve">{华能青岛项目}</t>
+          <t xml:space="preserve">{智慧家园项目}</t>
         </is>
       </c>
     </row>
@@ -8136,17 +8277,17 @@
       <c r="A29"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">华夏华润电力燃煤发电</t>
+          <t xml:space="preserve">中信建投广州发展清洁能源</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">华润电力控股有限公司</t>
+          <t xml:space="preserve">广州产业投资控股集团有限公司</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">华润焦作电厂项目</t>
+          <t xml:space="preserve">东明东南风电项目、东明西南一期风电项目、东明西南二期风电项目</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -8161,17 +8302,17 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">焦作市</t>
+          <t xml:space="preserve">菏泽市</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">河南省</t>
+          <t xml:space="preserve">山东省</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t xml:space="preserve">{华润焦作电厂项目}</t>
+          <t xml:space="preserve">{东明东南风电项目，东明西南一期风电项目，东明西南二期风电项目}</t>
         </is>
       </c>
     </row>
@@ -8179,42 +8320,42 @@
       <c r="A30"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">华夏蜀道集团高速公路</t>
+          <t xml:space="preserve">招商资管招商蛇口</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">蜀道投资集团有限责任公司</t>
+          <t xml:space="preserve">招商蛇口工业区控股股份有限公司</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">雅泸高速公路项目</t>
+          <t xml:space="preserve">昆山招商花园城项目、深圳太子广场项目</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">基础设施REITs</t>
+          <t xml:space="preserve">商业不动产REITs</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">交通基础设施</t>
+          <t xml:space="preserve">办公+商业零售</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">雅安市，凉山彝族自治州</t>
+          <t xml:space="preserve">昆山市，深圳市</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">四川省，四川省</t>
+          <t xml:space="preserve">江苏省，广东省</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t xml:space="preserve">{雅泸高速公路项目}|{雅泸高速公路项目}</t>
+          <t xml:space="preserve">{昆山招商花园城项目}|{深圳太子广场项目}</t>
         </is>
       </c>
     </row>
@@ -8222,17 +8363,17 @@
       <c r="A31"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">华夏龙岗城投产业园</t>
+          <t xml:space="preserve">博时招商蛇口产业园（扩募）</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">深圳市龙岗区城市建设投资集团有限公司</t>
+          <t xml:space="preserve">招商蛇口工业区控股股份有限公司</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">智慧家园项目</t>
+          <t xml:space="preserve">光明项目（二期扩募）、南油项目</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -8242,7 +8383,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">园区基础设施</t>
+          <t xml:space="preserve">产业园+仓储物流</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -8257,7 +8398,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t xml:space="preserve">{智慧家园项目}</t>
+          <t xml:space="preserve">{光明项目（二期扩募），南油项目}</t>
         </is>
       </c>
     </row>
@@ -8265,42 +8406,42 @@
       <c r="A32"/>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">中信建投广州发展清洁能源</t>
+          <t xml:space="preserve">广发海珠城发</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">广州产业投资控股集团有限公司</t>
+          <t xml:space="preserve">广州市海珠城市建设发展集团有限公司</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">东明东南风电项目、东明西南一期风电项目、东明西南二期风电项目</t>
+          <t xml:space="preserve">广州朗豪酒店</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">基础设施REITs</t>
+          <t xml:space="preserve">商业不动产REITs</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">能源基础设施</t>
+          <t xml:space="preserve">酒店</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">菏泽市</t>
+          <t xml:space="preserve">广州市</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">山东省</t>
+          <t xml:space="preserve">广东省</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t xml:space="preserve">{东明东南风电项目，东明西南一期风电项目，东明西南二期风电项目}</t>
+          <t xml:space="preserve">{广州朗豪酒店}</t>
         </is>
       </c>
     </row>
@@ -8308,42 +8449,42 @@
       <c r="A33"/>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">招商资管招商蛇口</t>
+          <t xml:space="preserve">东方红申能股份新能源</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">招商蛇口工业区控股股份有限公司</t>
+          <t xml:space="preserve">申能股份有限公司</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">昆山招商花园城项目、深圳太子广场项目</t>
+          <t xml:space="preserve">乌兰20万千瓦风电项目</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业不动产REITs</t>
+          <t xml:space="preserve">基础设施REITs</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">办公+商业零售</t>
+          <t xml:space="preserve">能源基础设施</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">昆山市，深圳市</t>
+          <t xml:space="preserve">海西蒙古族藏族自治州</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">江苏省，广东省</t>
+          <t xml:space="preserve">青海省</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t xml:space="preserve">{昆山招商花园城项目}|{深圳太子广场项目}</t>
+          <t xml:space="preserve">{乌兰20万千瓦风电项目}</t>
         </is>
       </c>
     </row>
@@ -8351,17 +8492,17 @@
       <c r="A34"/>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">博时招商蛇口产业园（扩募）</t>
+          <t xml:space="preserve">南方润泽科技数据中心（扩募）</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">招商蛇口工业区控股股份有限公司</t>
+          <t xml:space="preserve">润泽智算科技集团股份有限公司</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">光明项目（二期扩募）、南油项目</t>
+          <t xml:space="preserve">A-7数据中心，A-8数据中心 </t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -8371,22 +8512,22 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">产业园+仓储物流</t>
+          <t xml:space="preserve">新型基础设施</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">深圳市</t>
+          <t xml:space="preserve">廊坊市</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">广东省</t>
+          <t xml:space="preserve">河北省</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t xml:space="preserve">{光明项目（二期扩募），南油项目}</t>
+          <t xml:space="preserve">{A-7数据中心，A-8数据中心 }</t>
         </is>
       </c>
     </row>
@@ -8394,17 +8535,17 @@
       <c r="A35"/>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">广发海珠城发</t>
+          <t xml:space="preserve">华夏大悦城</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">广州市海珠城市建设发展集团有限公司</t>
+          <t xml:space="preserve">中粮集团有限公司</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">广州朗豪酒店</t>
+          <t xml:space="preserve">天津大悦城项目</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -8414,22 +8555,22 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">酒店</t>
+          <t xml:space="preserve">商业零售</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">广州市</t>
+          <t xml:space="preserve">天津市</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve">广东省</t>
+          <t xml:space="preserve">天津市</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t xml:space="preserve">{广州朗豪酒店}</t>
+          <t xml:space="preserve">{天津大悦城项目}</t>
         </is>
       </c>
     </row>
@@ -8437,42 +8578,42 @@
       <c r="A36"/>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">东方红申能股份新能源</t>
+          <t xml:space="preserve">华泰紫金金鹰</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">申能股份有限公司</t>
+          <t xml:space="preserve">金鹰国际商贸集团（中国）有限公司</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">乌兰20万千瓦风电项目</t>
+          <t xml:space="preserve">金鹰湖滨天地（包含一期奥莱项目和二期购物中心项目）</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">基础设施REITs</t>
+          <t xml:space="preserve">商业不动产REITs</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">能源基础设施</t>
+          <t xml:space="preserve">奥特莱斯+商业零售</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">海西蒙古族藏族自治州</t>
+          <t xml:space="preserve">南京市</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t xml:space="preserve">青海省</t>
+          <t xml:space="preserve">江苏省</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t xml:space="preserve">{乌兰20万千瓦风电项目}</t>
+          <t xml:space="preserve">{金鹰湖滨天地一期奥莱项目，金鹰湖滨天地二期购物中心项目}</t>
         </is>
       </c>
     </row>
@@ -8480,42 +8621,42 @@
       <c r="A37"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">南方润泽科技数据中心（扩募）</t>
+          <t xml:space="preserve">华安中电浦软</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">润泽智算科技集团股份有限公司</t>
+          <t xml:space="preserve">中国电子信息产业集团有限公司</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">A-7数据中心，A-8数据中心 </t>
+          <t xml:space="preserve">上海汇智国际商业中心</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">基础设施REITs</t>
+          <t xml:space="preserve">商业不动产REITs</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">新型基础设施</t>
+          <t xml:space="preserve">商业零售</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">廊坊市</t>
+          <t xml:space="preserve">上海市</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t xml:space="preserve">河北省</t>
+          <t xml:space="preserve">上海市</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t xml:space="preserve">{A-7数据中心，A-8数据中心 }</t>
+          <t xml:space="preserve">{上海汇智国际商业中心}</t>
         </is>
       </c>
     </row>
@@ -8523,42 +8664,42 @@
       <c r="A38"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">华夏大悦城</t>
+          <t xml:space="preserve">嘉实京东仓储物流（扩募）</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">中粮集团有限公司</t>
+          <t xml:space="preserve">京东集团股份有限公司</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">天津大悦城项目</t>
+          <t xml:space="preserve">京东西北电子商务营业中心（京东二期）项目、京东安徽电子商务产业园二期项目</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业不动产REITs</t>
+          <t xml:space="preserve">基础设施REITs</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业零售</t>
+          <t xml:space="preserve">仓储物流基础设施</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">天津市</t>
+          <t xml:space="preserve">西安市，合肥市</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">天津市</t>
+          <t xml:space="preserve">陕西省，安徽省</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t xml:space="preserve">{天津大悦城项目}</t>
+          <t xml:space="preserve">{京东西北电子商务营业中心（京东二期）项目}|{京东安徽电子商务产业园二期项目}</t>
         </is>
       </c>
     </row>
@@ -8566,42 +8707,42 @@
       <c r="A39"/>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">华泰紫金金鹰</t>
+          <t xml:space="preserve">中金温州公用水利</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">金鹰国际商贸集团（中国）有限公司</t>
+          <t xml:space="preserve">温州市公用事业发展集团有限公司</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">金鹰湖滨天地（包含一期奥莱项目和二期购物中心项目）</t>
+          <t xml:space="preserve">温州市珊溪水利枢纽工程项目</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业不动产REITs</t>
+          <t xml:space="preserve">基础设施REITs</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">奥特莱斯+商业零售</t>
+          <t xml:space="preserve">水利基础设施</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">南京市</t>
+          <t xml:space="preserve">温州市</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve">江苏省</t>
+          <t xml:space="preserve">浙江省</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t xml:space="preserve">{金鹰湖滨天地一期奥莱项目，金鹰湖滨天地二期购物中心项目}</t>
+          <t xml:space="preserve">{温州市珊溪水利枢纽工程项目}</t>
         </is>
       </c>
     </row>
@@ -8609,42 +8750,42 @@
       <c r="A40"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">华安中电浦软</t>
+          <t xml:space="preserve">嘉实陶邑消费</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">中国电子信息产业集团有限公司</t>
+          <t xml:space="preserve">景德镇陶文旅控股集团有限公司</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">上海汇智国际商业中心</t>
+          <t xml:space="preserve">景德镇陶溪川首期项目</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业不动产REITs</t>
+          <t xml:space="preserve">基础设施REITs</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业零售</t>
+          <t xml:space="preserve">文旅基础设施</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">上海市</t>
+          <t xml:space="preserve">景德镇市</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">上海市</t>
+          <t xml:space="preserve">江西省</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t xml:space="preserve">{上海汇智国际商业中心}</t>
+          <t xml:space="preserve">{景德镇陶溪川首期项目}</t>
         </is>
       </c>
     </row>
@@ -8652,42 +8793,42 @@
       <c r="A41"/>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">嘉实京东仓储物流（扩募）</t>
+          <t xml:space="preserve">中金中国绿发</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">京东集团股份有限公司</t>
+          <t xml:space="preserve">中国绿发投资集团有限公司</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">京东西北电子商务营业中心（京东二期）项目、京东安徽电子商务产业园二期项目</t>
+          <t xml:space="preserve">济南贵和购物中心及贵和洲际酒店、上海艾迪逊酒店</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">基础设施REITs</t>
+          <t xml:space="preserve">商业不动产REITs</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">仓储物流基础设施</t>
+          <t xml:space="preserve">酒店+商业零售</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">西安市，合肥市</t>
+          <t xml:space="preserve">济南市，上海市</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve">陕西省，安徽省</t>
+          <t xml:space="preserve">山东省，上海市</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t xml:space="preserve">{京东西北电子商务营业中心（京东二期）项目}|{京东安徽电子商务产业园二期项目}</t>
+          <t xml:space="preserve">{济南贵和购物中心，贵和洲际酒店}|{上海艾迪逊酒店}</t>
         </is>
       </c>
     </row>
@@ -8695,42 +8836,42 @@
       <c r="A42"/>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">中金温州公用水利</t>
+          <t xml:space="preserve">华夏中海</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">温州市公用事业发展集团有限公司</t>
+          <t xml:space="preserve">中国海外集团有限公司</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">温州市珊溪水利枢纽工程项目</t>
+          <t xml:space="preserve">佛山千灯湖环宇城</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">基础设施REITs</t>
+          <t xml:space="preserve">商业不动产REITs</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">水利基础设施</t>
+          <t xml:space="preserve">商业零售</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">温州市</t>
+          <t xml:space="preserve">佛山市</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">浙江省</t>
+          <t xml:space="preserve">广东省</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t xml:space="preserve">{温州市珊溪水利枢纽工程项目}</t>
+          <t xml:space="preserve">{佛山千灯湖环宇城}</t>
         </is>
       </c>
     </row>
@@ -8738,17 +8879,17 @@
       <c r="A43"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">嘉实陶邑消费</t>
+          <t xml:space="preserve">国泰海通上实租赁住房</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">景德镇陶文旅控股集团有限公司</t>
+          <t xml:space="preserve">上海（上实）集团有限公司</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">景德镇陶溪川首期项目</t>
+          <t xml:space="preserve">上海城开·阡集汇社区</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -8758,22 +8899,22 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅基础设施</t>
+          <t xml:space="preserve">保障性租赁住房</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">景德镇市</t>
+          <t xml:space="preserve">上海市</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve">江西省</t>
+          <t xml:space="preserve">上海市</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t xml:space="preserve">{景德镇陶溪川首期项目}</t>
+          <t xml:space="preserve">{上海城开·阡集汇社区}</t>
         </is>
       </c>
     </row>
@@ -8781,17 +8922,17 @@
       <c r="A44"/>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">中金中国绿发</t>
+          <t xml:space="preserve">国联安泰华城</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">中国绿发投资集团有限公司</t>
+          <t xml:space="preserve">山东世纪泰华集团有限公司</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">济南贵和购物中心及贵和洲际酒店、上海艾迪逊酒店</t>
+          <t xml:space="preserve">潍坊泰华城项目，青州泰华城项目</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -8801,22 +8942,366 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">酒店+商业零售</t>
+          <t xml:space="preserve">商业零售</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">济南市，上海市</t>
+          <t xml:space="preserve">潍坊市，青州市</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">山东省，上海市</t>
+          <t xml:space="preserve">山东省，山东省</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t xml:space="preserve">{济南贵和购物中心，贵和洲际酒店}|{上海艾迪逊酒店}</t>
+          <t xml:space="preserve">{潍坊泰华城项目}|{青州泰华城项目}</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A45"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华安晶澳科技新能源</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">晶澳太阳能科技股份有限公司</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">河北省张家口市康保项目，辽宁省朝阳市朝阳项目</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">基础设施REITs</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">能源基础设施</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">张家口市，朝阳市</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">河北省，辽宁省</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{河北省张家口市康保项目}|{辽宁省朝阳市朝阳项目}</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A46"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国泰海通鹏瑞利</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PerennialGroupPrivateLimited</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">成都鹏瑞利青羊项目</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商业不动产REITs</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商业零售</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">成都市</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">四川省</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{成都鹏瑞利青羊项目}</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A47"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">广发新世界</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新世界发展有限公司</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上海新世界大厦（K11购物艺术中心）项目</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商业不动产REITs</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商业零售</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上海市</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上海市</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{上海新世界大厦（K11购物艺术中心）项目}</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A48"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华夏世纪金源</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">世纪金源投资集团有限公司</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合肥滨湖方圆荟项目</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商业不动产REITs</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商业零售</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">合肥市</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">安徽省</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{合肥滨湖方圆荟项目}</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A49"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国泰海通信义能源新能源</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">信义能源控股有限公司</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">芜湖市三山经济开发区100MW光伏电站项目、金寨县小南京村150MW光伏电站项目</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">基础设施REITs</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">能源基础设施</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">芜湖市，六安市</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">安徽省，安徽省</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{芜湖市三山经济开发区100MW光伏电站项目}|{金寨县小南京村150MW光伏电站项目}</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A50"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华夏凯华</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">凯华集团有限公司</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">广州国际轻纺城AB区项目</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商业不动产REITs</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">专业市场</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">广州市</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">广东省</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{广州国际轻纺城AB区项目}</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A51"/>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">汇添富顺联</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">佛山市顺联集团有限公司</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">顺联广场综合体、顺联机械城、顺联奥莱购物中心</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商业不动产REITs</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">商业零售+专业市场+奥特莱斯</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">佛山市</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">广东省</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{顺联广场综合体，顺联机械城，顺联奥莱购物中心}</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="2:9" ns1:dyDescent="0.25">
+      <c r="A52"/>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">汇添富上海地产租赁住房（扩募）</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上海地产（集团）有限公司</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">璟耀项目、璟博项目</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">基础设施REITs</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">保障性租赁住房</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上海市</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">上海市</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{璟耀项目，璟博项目}</t>
         </is>
       </c>
     </row>

</xml_diff>